<commit_message>
Verify official channels and contact portals for all 55 governors
</commit_message>
<xml_diff>
--- a/data/contacts.xlsx
+++ b/data/contacts.xlsx
@@ -4175,7 +4175,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.alabama.gov/contact/</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://gov.alaska.gov/contact/</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -4257,7 +4257,7 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -4319,7 +4319,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.americansamoa.gov/governorpulaalii</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -4329,7 +4329,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://azgovernor.gov/contact</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -4401,7 +4401,7 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.arkansas.gov/contact-the-governor/</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -4473,7 +4473,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.gov.ca.gov/contact/</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -4545,7 +4545,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -4597,7 +4597,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Governorpolis@state.co.us</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governorsoffice.colorado.gov/governor/contact-us</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -4617,7 +4617,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://portal.ct.gov/governor/contact/email-governor-lamont</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -4689,7 +4689,7 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.delaware.gov/contact-the-governors-office/</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.flgov.com/contact-governor/</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -4833,7 +4833,7 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -4895,7 +4895,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://gov.georgia.gov/contact-us</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -4905,7 +4905,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -4967,7 +4967,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.guam.gov/contact-us/</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -4977,7 +4977,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -5039,7 +5039,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.hawaii.gov/contact-us/</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -5049,7 +5049,7 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5111,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://gov.idaho.gov/contact-us/</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -5121,7 +5121,7 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://gov.illinois.gov/contact-us/</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.in.gov/gov/contact/</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -5327,7 +5327,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.iowa.gov/contact</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -5399,7 +5399,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.kansas.gov/contact/</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -5409,7 +5409,7 @@
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -5471,7 +5471,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.ky.gov/contact</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -5543,7 +5543,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://gov.louisiana.gov/page/contact</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -5553,7 +5553,7 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -5615,7 +5615,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.maine.gov/governor/mills/contact</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -5625,7 +5625,7 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -5687,7 +5687,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.maryland.gov/leadership/governor-wes-moore</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -5697,7 +5697,7 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -5759,7 +5759,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.mass.gov/info-details/email-the-governors-office</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -5769,7 +5769,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -5831,7 +5831,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.michigan.gov/whitmer/contact</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
@@ -5841,7 +5841,7 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -5903,7 +5903,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://mn.gov/governor/contact/</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
@@ -5913,7 +5913,7 @@
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -5975,7 +5975,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governorreeves.ms.gov/contact/</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
@@ -5985,7 +5985,7 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -6047,7 +6047,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.mo.gov/contact-us</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
@@ -6057,7 +6057,7 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -6119,7 +6119,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.mt.gov/Contact/default</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -6191,7 +6191,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.nebraska.gov/contact-form</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -6263,7 +6263,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://gov.nv.gov/Contact/Contact_Us/</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -6273,7 +6273,7 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -6335,7 +6335,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.governor.nh.gov/contact-us</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
@@ -6345,7 +6345,7 @@
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -6407,7 +6407,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.nj.gov/governor/contact/</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
@@ -6417,7 +6417,7 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -6479,7 +6479,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.governor.state.nm.us/contact-the-governor/</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
@@ -6489,7 +6489,7 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.governor.ny.gov/content/governor-contact-form</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
@@ -6561,7 +6561,7 @@
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -6623,7 +6623,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.nc.gov/contact</t>
         </is>
       </c>
       <c r="M92" t="inlineStr">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -6695,7 +6695,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.governor.nd.gov/contact-us</t>
         </is>
       </c>
       <c r="M93" t="inlineStr">
@@ -6705,7 +6705,7 @@
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -6767,7 +6767,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.cnmi.gov/contact/</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
@@ -6777,7 +6777,7 @@
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -6839,7 +6839,7 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.ohio.gov/contact</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
@@ -6849,7 +6849,7 @@
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -6911,7 +6911,7 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://oklahoma.gov/governor/contact.html</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
@@ -6921,7 +6921,7 @@
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -6983,7 +6983,7 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.oregon.gov/gov/Pages/share-your-opinion.aspx</t>
         </is>
       </c>
       <c r="M97" t="inlineStr">
@@ -6993,7 +6993,7 @@
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -7055,7 +7055,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.governor.pa.gov/contact/</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
@@ -7065,7 +7065,7 @@
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -7127,7 +7127,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.fortaleza.pr.gov/</t>
         </is>
       </c>
       <c r="M99" t="inlineStr">
@@ -7137,7 +7137,7 @@
       </c>
       <c r="N99" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -7199,7 +7199,7 @@
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.ri.gov/contact-us</t>
         </is>
       </c>
       <c r="M100" t="inlineStr">
@@ -7209,7 +7209,7 @@
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -7271,7 +7271,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.sc.gov/contact-office-governor</t>
         </is>
       </c>
       <c r="M101" t="inlineStr">
@@ -7281,7 +7281,7 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -7343,7 +7343,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.sd.gov/contact.aspx</t>
         </is>
       </c>
       <c r="M102" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -7415,7 +7415,7 @@
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.tn.gov/governor/contact-us.html</t>
         </is>
       </c>
       <c r="M103" t="inlineStr">
@@ -7425,7 +7425,7 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -7487,7 +7487,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://gov.texas.gov/contact</t>
         </is>
       </c>
       <c r="M104" t="inlineStr">
@@ -7497,7 +7497,7 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -7559,7 +7559,7 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.utah.gov/contact/</t>
         </is>
       </c>
       <c r="M105" t="inlineStr">
@@ -7569,7 +7569,7 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -7631,7 +7631,7 @@
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.vermont.gov/contact-us</t>
         </is>
       </c>
       <c r="M106" t="inlineStr">
@@ -7641,7 +7641,7 @@
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -7703,7 +7703,7 @@
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.vi.gov/governor-bryan/</t>
         </is>
       </c>
       <c r="M107" t="inlineStr">
@@ -7713,7 +7713,7 @@
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -7775,7 +7775,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.governor.virginia.gov/constituent-services/contact-the-governor/</t>
         </is>
       </c>
       <c r="M108" t="inlineStr">
@@ -7785,7 +7785,7 @@
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -7847,7 +7847,7 @@
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.wa.gov/contacting-governor/contacting-governors-office</t>
         </is>
       </c>
       <c r="M109" t="inlineStr">
@@ -7857,7 +7857,7 @@
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -7919,7 +7919,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.wv.gov/Pages/Contact.aspx</t>
         </is>
       </c>
       <c r="M110" t="inlineStr">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -7991,7 +7991,7 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://evers.wi.gov/pages/connect.aspx</t>
         </is>
       </c>
       <c r="M111" t="inlineStr">
@@ -8001,7 +8001,7 @@
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -8063,7 +8063,7 @@
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.wyo.gov/contact</t>
         </is>
       </c>
       <c r="M112" t="inlineStr">
@@ -8073,7 +8073,7 @@
       </c>
       <c r="N112" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -8208,12 +8208,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.alabama.gov/contact/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора. Связь через веб-форму и приёмную; прямой публичный email и LinkedIn не публикуются.</t>
         </is>
       </c>
     </row>
@@ -8260,12 +8260,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://gov.alaska.gov/contact/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -8275,7 +8275,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора. Связь через официальную форму обращений; прямой email и LinkedIn не публикуются.</t>
         </is>
       </c>
     </row>
@@ -8312,12 +8312,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.americansamoa.gov/governorpulaalii</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -8327,7 +8327,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный правительственный портал Американского Самоа. Связь через аппарат губернатора; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -8364,12 +8364,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://azgovernor.gov/contact</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -8379,7 +8379,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт офиса губернатора. Связь через защищённую форму обращений граждан; прямой email и LinkedIn не публикуются.</t>
         </is>
       </c>
     </row>
@@ -8416,12 +8416,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.arkansas.gov/contact-the-governor/</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -8431,7 +8431,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт губернатора. Связь через веб-форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -8468,12 +8468,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.gov.ca.gov/contact/</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -8483,7 +8483,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Калифорнии. Связь через онлайн-форму приёмной; прямой email и личный LinkedIn не публикуются.</t>
         </is>
       </c>
     </row>
@@ -8520,12 +8520,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governorsoffice.colorado.gov/governor/contact-us</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -8535,7 +8535,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал офиса губернатора. Опубликован официальный служебный адрес электронной почты Governorpolis@state.co.us.</t>
         </is>
       </c>
     </row>
@@ -8572,12 +8572,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://portal.ct.gov/governor/contact/email-governor-lamont</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -8587,7 +8587,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал штата Коннектикут. Связь через форму обращений граждан; прямой публичный email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -8624,12 +8624,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.delaware.gov/contact-the-governors-office/</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -8639,7 +8639,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Делавэра. Связь через форму обращений и телефонную линию; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -8676,12 +8676,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.flgov.com/contact-governor/</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал Executive Office of the Governor. Связь через контактную форму; прямой публичный email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -8728,12 +8728,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://gov.georgia.gov/contact-us</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -8743,7 +8743,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Джорджии. Связь через форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -8780,12 +8780,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.guam.gov/contact-us/</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -8795,7 +8795,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт офиса губернатора Гуама. Связь через контактную страницу и приёмную; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -8832,12 +8832,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.hawaii.gov/contact-us/</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -8847,7 +8847,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт губернатора Гавайев. Связь через веб-форму и канцелярию; прямой публичный email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -8884,12 +8884,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://gov.idaho.gov/contact-us/</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -8899,7 +8899,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Айдахо. Связь через форму обращения граждан; прямой подтверждённый email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -8936,12 +8936,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://gov.illinois.gov/contact-us/</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -8951,7 +8951,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт губернатора Иллинойса. Связь через веб-форму обращений; прямой публичный email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -8988,12 +8988,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.in.gov/gov/contact/</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -9003,7 +9003,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Индианы. Связь через защищённую онлайн-форму IN.gov; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9040,12 +9040,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.iowa.gov/contact</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -9055,7 +9055,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Айовы. Связь через онлайн-форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9092,12 +9092,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.kansas.gov/contact/</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -9107,7 +9107,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт губернатора Канзаса. Связь через портал обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9144,12 +9144,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.ky.gov/contact</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -9159,7 +9159,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Кентукки. Связь через форму обращений граждан; прямой публичный email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9196,12 +9196,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://gov.louisiana.gov/page/contact</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -9211,7 +9211,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт офиса губернатора Луизианы. Связь через контактную веб-форму; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9248,12 +9248,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.maine.gov/governor/mills/contact</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -9263,7 +9263,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора штата Мэн. Связь через онлайн-форму обращений граждан; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9300,12 +9300,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.maryland.gov/leadership/governor-wes-moore</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -9315,7 +9315,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Мэриленда. Связь через канцелярию и веб-портал; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9352,12 +9352,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.mass.gov/info-details/email-the-governors-office</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -9367,7 +9367,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал Содружества Массачусетс. Связь через форму Email the Governor Office; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9404,12 +9404,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.michigan.gov/whitmer/contact</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -9419,7 +9419,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Мичигана. Связь через форму службы поддержки граждан; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9456,12 +9456,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://mn.gov/governor/contact/</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Миннесоты. Связь через онлайн-форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9508,12 +9508,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governorreeves.ms.gov/contact/</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -9523,7 +9523,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт губернатора Миссисипи. Связь через контактную форму; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9560,12 +9560,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.mo.gov/contact-us</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -9575,7 +9575,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Миссури. Связь через контактную онлайн-форму; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9612,12 +9612,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.mt.gov/Contact/default</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -9627,7 +9627,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт губернатора Монтаны. Связь через веб-форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9664,12 +9664,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.nebraska.gov/contact-form</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -9679,7 +9679,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт губернатора Небраски. Связь через форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9716,12 +9716,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://gov.nv.gov/Contact/Contact_Us/</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -9731,7 +9731,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Невады. Связь через контактную форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9768,12 +9768,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.governor.nh.gov/contact-us</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -9783,7 +9783,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Нью-Гэмпшира. Связь через веб-форму и канцелярию; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9820,12 +9820,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.nj.gov/governor/contact/</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -9835,7 +9835,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Нью-Джерси. Связь через онлайн-форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9872,12 +9872,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.governor.state.nm.us/contact-the-governor/</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -9887,7 +9887,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Нью-Мексико. Связь через форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9924,12 +9924,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.governor.ny.gov/content/governor-contact-form</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -9939,7 +9939,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Нью-Йорка. Связь через электронную контактную форму; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -9976,12 +9976,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.nc.gov/contact</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -9991,7 +9991,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Северной Каролины. Связь через контактную веб-форму; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10028,12 +10028,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.governor.nd.gov/contact-us</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -10043,7 +10043,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Северной Дакоты. Связь через контактную форму; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10080,12 +10080,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.cnmi.gov/contact/</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -10095,7 +10095,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора СМОИ. Связь через контактную форму и канцелярию; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10132,12 +10132,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.ohio.gov/contact</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -10147,7 +10147,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Огайо. Связь через веб-форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10184,12 +10184,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://oklahoma.gov/governor/contact.html</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -10199,7 +10199,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал штата Оклахома. Связь через контактную форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10236,12 +10236,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.oregon.gov/gov/Pages/share-your-opinion.aspx</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Орегона. Связь через веб-форму обращений граждан; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10288,12 +10288,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.governor.pa.gov/contact/</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -10303,7 +10303,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Пенсильвании. Связь через онлайн-форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10340,12 +10340,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.fortaleza.pr.gov/</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -10355,7 +10355,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал администрации губернатора Пуэрто-Рико (La Fortaleza). Связь через канцелярию; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10392,12 +10392,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.ri.gov/contact-us</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -10407,7 +10407,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт губернатора Род-Айленда. Связь через онлайн-форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10444,12 +10444,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.sc.gov/contact-office-governor</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -10459,7 +10459,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт губернатора Южной Каролины. Связь через форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10496,12 +10496,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.sd.gov/contact.aspx</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -10511,7 +10511,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт губернатора Южной Дакоты. Связь через веб-форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10548,12 +10548,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.tn.gov/governor/contact-us.html</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -10563,7 +10563,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал штата Теннесси. Связь через форму Share My Opinion; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10600,12 +10600,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://gov.texas.gov/contact</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -10615,7 +10615,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Техаса. Связь через защищённую контактную форму и телефонные линии; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10652,12 +10652,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.utah.gov/contact/</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -10667,7 +10667,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт губернатора Юты. Связь через форму обращений граждан; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10704,12 +10704,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.vermont.gov/contact-us</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Вермонта. Связь через онлайн-форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10756,12 +10756,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.vi.gov/governor-bryan/</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -10771,7 +10771,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал правительства Американских Виргинских Островов. Связь через канцелярию губернатора; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10808,12 +10808,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://www.governor.virginia.gov/constituent-services/contact-the-governor/</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -10823,7 +10823,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт губернатора Виргинии. Связь через портал Constituent Services; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10860,12 +10860,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.wa.gov/contacting-governor/contacting-governors-office</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -10875,7 +10875,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Вашингтона. Связь через электронную форму обращений; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10912,12 +10912,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.wv.gov/Pages/Contact.aspx</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -10927,7 +10927,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Западной Виргинии. Связь через контактную веб-форму; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -10964,12 +10964,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://evers.wi.gov/pages/connect.aspx</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -10979,7 +10979,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный сайт губернатора Висконсина. Связь через портал Connect with the Governor; прямой email не публикуется.</t>
         </is>
       </c>
     </row>
@@ -11016,12 +11016,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t xml:space="preserve">in_progress</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.nga.org/Governors/</t>
+          <t xml:space="preserve">https://governor.wyo.gov/contact</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -11031,7 +11031,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя взято из текущего списка NGA; служебная почта и LinkedIn требуют отдельной проверки.</t>
+          <t xml:space="preserve">Официальный портал губернатора Вайоминга. Связь через форму обращений и телефонную связь; прямой email не публикуется.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add offline dataset validator with tests, label uncovered roles as not_started, verify sample leads
The validator checks format only (email syntax, NANP phone when a phone
column exists, source URLs, dates, duplicates) and keeps format checks
separate from proof that an inbox or number is active. 540 not_started
coverage rows keep uncovered roles visibly empty; Alabama and DC leads
are corrected against official agency pages; dist and workbook rebuilt
for 172 contacts.
</commit_message>
<xml_diff>
--- a/data/contacts.xlsx
+++ b/data/contacts.xlsx
@@ -108,7 +108,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Foreign Affairs Officer/FDI Manager</t>
+          <t xml:space="preserve">Foreign Affairs Officer/FDI</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -153,7 +153,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.trade.gov/selectusa-find-economic-developers</t>
+          <t xml:space="preserve">https://www.madeinalabama.com/resources/contacts/gary-walton/</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -163,7 +163,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Director of Business Attraction</t>
+          <t xml:space="preserve">Vice President of International Business Attraction</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Office of the Deputy Mayor for Planning and Economic Development</t>
+          <t xml:space="preserve">Washington DC Economic Partnership</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.trade.gov/selectusa-find-economic-developers</t>
+          <t xml:space="preserve">https://wdcep.com/team/</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_review</t>
+          <t xml:space="preserve">verified</t>
         </is>
       </c>
     </row>

</xml_diff>